<commit_message>
Avancement des exercices de la partie 1.
</commit_message>
<xml_diff>
--- a/Maths/Moteur_RTS_amelioration_modele_population.xlsx
+++ b/Maths/Moteur_RTS_amelioration_modele_population.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trist\Desktop\moteur_RTS\Maths\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B01E01-676B-4CA2-B35C-A6A71BAF5A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07F52E3-E4D9-41E8-B294-395B0A038135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2B550C33-22D4-41CD-BFC0-2BCA21971097}"/>
+    <workbookView xWindow="3072" yWindow="3072" windowWidth="17280" windowHeight="9420" xr2:uid="{2B550C33-22D4-41CD-BFC0-2BCA21971097}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -50,13 +50,13 @@
     <t>Temps (jours après le début de la simulation)</t>
   </si>
   <si>
-    <t>Const K (population initiale)</t>
-  </si>
-  <si>
     <t>Const a (Taux de reproduction)</t>
   </si>
   <si>
     <t>Const b (taux de mortalité)</t>
+  </si>
+  <si>
+    <t>Const K</t>
   </si>
 </sst>
 </file>
@@ -4239,1601 +4239,1001 @@
           </cell>
         </row>
         <row r="3">
-          <cell r="A3">
-            <v>2.0000200001000001</v>
-          </cell>
           <cell r="B3">
             <v>1</v>
           </cell>
         </row>
         <row r="4">
-          <cell r="A4">
-            <v>2.0000400004000025</v>
-          </cell>
           <cell r="B4">
             <v>2</v>
           </cell>
         </row>
         <row r="5">
-          <cell r="A5">
-            <v>2.0000600009000089</v>
-          </cell>
           <cell r="B5">
             <v>3</v>
           </cell>
         </row>
         <row r="6">
-          <cell r="A6">
-            <v>2.0000800016000215</v>
-          </cell>
           <cell r="B6">
             <v>4</v>
           </cell>
         </row>
         <row r="7">
-          <cell r="A7">
-            <v>2.0001000025000417</v>
-          </cell>
           <cell r="B7">
             <v>5</v>
           </cell>
         </row>
         <row r="8">
-          <cell r="A8">
-            <v>2.0001200036000721</v>
-          </cell>
           <cell r="B8">
             <v>6</v>
           </cell>
         </row>
         <row r="9">
-          <cell r="A9">
-            <v>2.0001400049001141</v>
-          </cell>
           <cell r="B9">
             <v>7</v>
           </cell>
         </row>
         <row r="10">
-          <cell r="A10">
-            <v>2.0001600064001708</v>
-          </cell>
           <cell r="B10">
             <v>8</v>
           </cell>
         </row>
         <row r="11">
-          <cell r="A11">
-            <v>2.000180008100243</v>
-          </cell>
           <cell r="B11">
             <v>9</v>
           </cell>
         </row>
         <row r="12">
-          <cell r="A12">
-            <v>2.0002000100003334</v>
-          </cell>
           <cell r="B12">
             <v>10</v>
           </cell>
         </row>
         <row r="13">
-          <cell r="A13">
-            <v>2.0002200121004439</v>
-          </cell>
           <cell r="B13">
             <v>11</v>
           </cell>
         </row>
         <row r="14">
-          <cell r="A14">
-            <v>2.0002400144005761</v>
-          </cell>
           <cell r="B14">
             <v>12</v>
           </cell>
         </row>
         <row r="15">
-          <cell r="A15">
-            <v>2.0002600169007323</v>
-          </cell>
           <cell r="B15">
             <v>13</v>
           </cell>
         </row>
         <row r="16">
-          <cell r="A16">
-            <v>2.0002800196009147</v>
-          </cell>
           <cell r="B16">
             <v>14</v>
           </cell>
         </row>
         <row r="17">
-          <cell r="A17">
-            <v>2.0003000225011252</v>
-          </cell>
           <cell r="B17">
             <v>15</v>
           </cell>
         </row>
         <row r="18">
-          <cell r="A18">
-            <v>2.0003200256013653</v>
-          </cell>
           <cell r="B18">
             <v>16</v>
           </cell>
         </row>
         <row r="19">
-          <cell r="A19">
-            <v>2.0003400289016375</v>
-          </cell>
           <cell r="B19">
             <v>17</v>
           </cell>
         </row>
         <row r="20">
-          <cell r="A20">
-            <v>2.0003600324019439</v>
-          </cell>
           <cell r="B20">
             <v>18</v>
           </cell>
         </row>
         <row r="21">
-          <cell r="A21">
-            <v>2.0003800361022863</v>
-          </cell>
           <cell r="B21">
             <v>19</v>
           </cell>
         </row>
         <row r="22">
-          <cell r="A22">
-            <v>2.0004000400026669</v>
-          </cell>
           <cell r="B22">
             <v>20</v>
           </cell>
         </row>
         <row r="23">
-          <cell r="A23">
-            <v>2.000420044103087</v>
-          </cell>
           <cell r="B23">
             <v>21</v>
           </cell>
         </row>
         <row r="24">
-          <cell r="A24">
-            <v>2.0004400484035494</v>
-          </cell>
           <cell r="B24">
             <v>22</v>
           </cell>
         </row>
         <row r="25">
-          <cell r="A25">
-            <v>2.0004600529040557</v>
-          </cell>
           <cell r="B25">
             <v>23</v>
           </cell>
         </row>
         <row r="26">
-          <cell r="A26">
-            <v>2.0004800576046082</v>
-          </cell>
           <cell r="B26">
             <v>24</v>
           </cell>
         </row>
         <row r="27">
-          <cell r="A27">
-            <v>2.0005000625052087</v>
-          </cell>
           <cell r="B27">
             <v>25</v>
           </cell>
         </row>
         <row r="28">
-          <cell r="A28">
-            <v>2.000520067605859</v>
-          </cell>
           <cell r="B28">
             <v>26</v>
           </cell>
         </row>
         <row r="29">
-          <cell r="A29">
-            <v>2.0005400729065617</v>
-          </cell>
           <cell r="B29">
             <v>27</v>
           </cell>
         </row>
         <row r="30">
-          <cell r="A30">
-            <v>2.0005600784073176</v>
-          </cell>
           <cell r="B30">
             <v>28</v>
           </cell>
         </row>
         <row r="31">
-          <cell r="A31">
-            <v>2.00058008410813</v>
-          </cell>
           <cell r="B31">
             <v>29</v>
           </cell>
         </row>
         <row r="32">
-          <cell r="A32">
-            <v>2.0006000900090006</v>
-          </cell>
           <cell r="B32">
             <v>30</v>
           </cell>
         </row>
         <row r="33">
-          <cell r="A33">
-            <v>2.0006200961099312</v>
-          </cell>
           <cell r="B33">
             <v>31</v>
           </cell>
         </row>
         <row r="34">
-          <cell r="A34">
-            <v>2.0006401024109235</v>
-          </cell>
           <cell r="B34">
             <v>32</v>
           </cell>
         </row>
         <row r="35">
-          <cell r="A35">
-            <v>2.0006601089119802</v>
-          </cell>
           <cell r="B35">
             <v>33</v>
           </cell>
         </row>
         <row r="36">
-          <cell r="A36">
-            <v>2.0006801156131027</v>
-          </cell>
           <cell r="B36">
             <v>34</v>
           </cell>
         </row>
         <row r="37">
-          <cell r="A37">
-            <v>2.0007001225142931</v>
-          </cell>
           <cell r="B37">
             <v>35</v>
           </cell>
         </row>
         <row r="38">
-          <cell r="A38">
-            <v>2.0007201296155532</v>
-          </cell>
           <cell r="B38">
             <v>36</v>
           </cell>
         </row>
         <row r="39">
-          <cell r="A39">
-            <v>2.0007401369168858</v>
-          </cell>
           <cell r="B39">
             <v>37</v>
           </cell>
         </row>
         <row r="40">
-          <cell r="A40">
-            <v>2.0007601444182925</v>
-          </cell>
           <cell r="B40">
             <v>38</v>
           </cell>
         </row>
         <row r="41">
-          <cell r="A41">
-            <v>2.0007801521197748</v>
-          </cell>
           <cell r="B41">
             <v>39</v>
           </cell>
         </row>
         <row r="42">
-          <cell r="A42">
-            <v>2.0008001600213356</v>
-          </cell>
           <cell r="B42">
             <v>40</v>
           </cell>
         </row>
         <row r="43">
-          <cell r="A43">
-            <v>2.000820168122976</v>
-          </cell>
           <cell r="B43">
             <v>41</v>
           </cell>
         </row>
         <row r="44">
-          <cell r="A44">
-            <v>2.0008401764246986</v>
-          </cell>
           <cell r="B44">
             <v>42</v>
           </cell>
         </row>
         <row r="45">
-          <cell r="A45">
-            <v>2.0008601849265051</v>
-          </cell>
           <cell r="B45">
             <v>43</v>
           </cell>
         </row>
         <row r="46">
-          <cell r="A46">
-            <v>2.0008801936283978</v>
-          </cell>
           <cell r="B46">
             <v>44</v>
           </cell>
         </row>
         <row r="47">
-          <cell r="A47">
-            <v>2.0009002025303784</v>
-          </cell>
           <cell r="B47">
             <v>45</v>
           </cell>
         </row>
         <row r="48">
-          <cell r="A48">
-            <v>2.0009202116324492</v>
-          </cell>
           <cell r="B48">
             <v>46</v>
           </cell>
         </row>
         <row r="49">
-          <cell r="A49">
-            <v>2.0009402209346119</v>
-          </cell>
           <cell r="B49">
             <v>47</v>
           </cell>
         </row>
         <row r="50">
-          <cell r="A50">
-            <v>2.0009602304368683</v>
-          </cell>
           <cell r="B50">
             <v>48</v>
           </cell>
         </row>
         <row r="51">
-          <cell r="A51">
-            <v>2.0009802401392212</v>
-          </cell>
           <cell r="B51">
             <v>49</v>
           </cell>
         </row>
         <row r="52">
-          <cell r="A52">
-            <v>2.0010002500416717</v>
-          </cell>
           <cell r="B52">
             <v>50</v>
           </cell>
         </row>
         <row r="53">
-          <cell r="A53">
-            <v>2.0010202601442226</v>
-          </cell>
           <cell r="B53">
             <v>51</v>
           </cell>
         </row>
         <row r="54">
-          <cell r="A54">
-            <v>2.0010402704468753</v>
-          </cell>
           <cell r="B54">
             <v>52</v>
           </cell>
         </row>
         <row r="55">
-          <cell r="A55">
-            <v>2.0010602809496323</v>
-          </cell>
           <cell r="B55">
             <v>53</v>
           </cell>
         </row>
         <row r="56">
-          <cell r="A56">
-            <v>2.001080291652495</v>
-          </cell>
           <cell r="B56">
             <v>54</v>
           </cell>
         </row>
         <row r="57">
-          <cell r="A57">
-            <v>2.0011003025554661</v>
-          </cell>
           <cell r="B57">
             <v>55</v>
           </cell>
         </row>
         <row r="58">
-          <cell r="A58">
-            <v>2.0011203136585469</v>
-          </cell>
           <cell r="B58">
             <v>56</v>
           </cell>
         </row>
         <row r="59">
-          <cell r="A59">
-            <v>2.0011403249617397</v>
-          </cell>
           <cell r="B59">
             <v>57</v>
           </cell>
         </row>
         <row r="60">
-          <cell r="A60">
-            <v>2.001160336465047</v>
-          </cell>
           <cell r="B60">
             <v>58</v>
           </cell>
         </row>
         <row r="61">
-          <cell r="A61">
-            <v>2.0011803481684698</v>
-          </cell>
           <cell r="B61">
             <v>59</v>
           </cell>
         </row>
         <row r="62">
-          <cell r="A62">
-            <v>2.0012003600720107</v>
-          </cell>
           <cell r="B62">
             <v>60</v>
           </cell>
         </row>
         <row r="63">
-          <cell r="A63">
-            <v>2.0012203721756721</v>
-          </cell>
           <cell r="B63">
             <v>61</v>
           </cell>
         </row>
         <row r="64">
-          <cell r="A64">
-            <v>2.0012403844794551</v>
-          </cell>
           <cell r="B64">
             <v>62</v>
           </cell>
         </row>
         <row r="65">
-          <cell r="A65">
-            <v>2.001260396983362</v>
-          </cell>
           <cell r="B65">
             <v>63</v>
           </cell>
         </row>
         <row r="66">
-          <cell r="A66">
-            <v>2.0012804096873955</v>
-          </cell>
           <cell r="B66">
             <v>64</v>
           </cell>
         </row>
         <row r="67">
-          <cell r="A67">
-            <v>2.0013004225915565</v>
-          </cell>
           <cell r="B67">
             <v>65</v>
           </cell>
         </row>
         <row r="68">
-          <cell r="A68">
-            <v>2.0013204356958476</v>
-          </cell>
           <cell r="B68">
             <v>66</v>
           </cell>
         </row>
         <row r="69">
-          <cell r="A69">
-            <v>2.0013404490002711</v>
-          </cell>
           <cell r="B69">
             <v>67</v>
           </cell>
         </row>
         <row r="70">
-          <cell r="A70">
-            <v>2.0013604625048287</v>
-          </cell>
           <cell r="B70">
             <v>68</v>
           </cell>
         </row>
         <row r="71">
-          <cell r="A71">
-            <v>2.0013804762095218</v>
-          </cell>
           <cell r="B71">
             <v>69</v>
           </cell>
         </row>
         <row r="72">
-          <cell r="A72">
-            <v>2.0014004901143534</v>
-          </cell>
           <cell r="B72">
             <v>70</v>
           </cell>
         </row>
         <row r="73">
-          <cell r="A73">
-            <v>2.0014205042193249</v>
-          </cell>
           <cell r="B73">
             <v>71</v>
           </cell>
         </row>
         <row r="74">
-          <cell r="A74">
-            <v>2.0014405185244386</v>
-          </cell>
           <cell r="B74">
             <v>72</v>
           </cell>
         </row>
         <row r="75">
-          <cell r="A75">
-            <v>2.0014605330296962</v>
-          </cell>
           <cell r="B75">
             <v>73</v>
           </cell>
         </row>
         <row r="76">
-          <cell r="A76">
-            <v>2.0014805477350999</v>
-          </cell>
           <cell r="B76">
             <v>74</v>
           </cell>
         </row>
         <row r="77">
-          <cell r="A77">
-            <v>2.0015005626406515</v>
-          </cell>
           <cell r="B77">
             <v>75</v>
           </cell>
         </row>
         <row r="78">
-          <cell r="A78">
-            <v>2.0015205777463532</v>
-          </cell>
           <cell r="B78">
             <v>76</v>
           </cell>
         </row>
         <row r="79">
-          <cell r="A79">
-            <v>2.0015405930522068</v>
-          </cell>
           <cell r="B79">
             <v>77</v>
           </cell>
         </row>
         <row r="80">
-          <cell r="A80">
-            <v>2.0015606085582149</v>
-          </cell>
           <cell r="B80">
             <v>78</v>
           </cell>
         </row>
         <row r="81">
-          <cell r="A81">
-            <v>2.001580624264379</v>
-          </cell>
           <cell r="B81">
             <v>79</v>
           </cell>
         </row>
         <row r="82">
-          <cell r="A82">
-            <v>2.0016006401707007</v>
-          </cell>
           <cell r="B82">
             <v>80</v>
           </cell>
         </row>
         <row r="83">
-          <cell r="A83">
-            <v>2.0016206562771828</v>
-          </cell>
           <cell r="B83">
             <v>81</v>
           </cell>
         </row>
         <row r="84">
-          <cell r="A84">
-            <v>2.0016406725838269</v>
-          </cell>
           <cell r="B84">
             <v>82</v>
           </cell>
         </row>
         <row r="85">
-          <cell r="A85">
-            <v>2.0016606890906354</v>
-          </cell>
           <cell r="B85">
             <v>83</v>
           </cell>
         </row>
         <row r="86">
-          <cell r="A86">
-            <v>2.0016807057976096</v>
-          </cell>
           <cell r="B86">
             <v>84</v>
           </cell>
         </row>
         <row r="87">
-          <cell r="A87">
-            <v>2.0017007227047516</v>
-          </cell>
           <cell r="B87">
             <v>85</v>
           </cell>
         </row>
         <row r="88">
-          <cell r="A88">
-            <v>2.0017207398120642</v>
-          </cell>
           <cell r="B88">
             <v>86</v>
           </cell>
         </row>
         <row r="89">
-          <cell r="A89">
-            <v>2.0017407571195487</v>
-          </cell>
           <cell r="B89">
             <v>87</v>
           </cell>
         </row>
         <row r="90">
-          <cell r="A90">
-            <v>2.0017607746272073</v>
-          </cell>
           <cell r="B90">
             <v>88</v>
           </cell>
         </row>
         <row r="91">
-          <cell r="A91">
-            <v>2.0017807923350421</v>
-          </cell>
           <cell r="B91">
             <v>89</v>
           </cell>
         </row>
         <row r="92">
-          <cell r="A92">
-            <v>2.0018008102430547</v>
-          </cell>
           <cell r="B92">
             <v>90</v>
           </cell>
         </row>
         <row r="93">
-          <cell r="A93">
-            <v>2.0018208283512475</v>
-          </cell>
           <cell r="B93">
             <v>91</v>
           </cell>
         </row>
         <row r="94">
-          <cell r="A94">
-            <v>2.0018408466596225</v>
-          </cell>
           <cell r="B94">
             <v>92</v>
           </cell>
         </row>
         <row r="95">
-          <cell r="A95">
-            <v>2.0018608651681813</v>
-          </cell>
           <cell r="B95">
             <v>93</v>
           </cell>
         </row>
         <row r="96">
-          <cell r="A96">
-            <v>2.0018808838769262</v>
-          </cell>
           <cell r="B96">
             <v>94</v>
           </cell>
         </row>
         <row r="97">
-          <cell r="A97">
-            <v>2.0019009027858594</v>
-          </cell>
           <cell r="B97">
             <v>95</v>
           </cell>
         </row>
         <row r="98">
-          <cell r="A98">
-            <v>2.0019209218949827</v>
-          </cell>
           <cell r="B98">
             <v>96</v>
           </cell>
         </row>
         <row r="99">
-          <cell r="A99">
-            <v>2.0019409412042983</v>
-          </cell>
           <cell r="B99">
             <v>97</v>
           </cell>
         </row>
         <row r="100">
-          <cell r="A100">
-            <v>2.0019609607138076</v>
-          </cell>
           <cell r="B100">
             <v>98</v>
           </cell>
         </row>
         <row r="101">
-          <cell r="A101">
-            <v>2.0019809804235131</v>
-          </cell>
           <cell r="B101">
             <v>99</v>
           </cell>
         </row>
         <row r="102">
-          <cell r="A102">
-            <v>2.0020010003334168</v>
-          </cell>
           <cell r="B102">
             <v>100</v>
           </cell>
         </row>
         <row r="103">
-          <cell r="A103">
-            <v>2.0020210204435203</v>
-          </cell>
           <cell r="B103">
             <v>101</v>
           </cell>
         </row>
         <row r="104">
-          <cell r="A104">
-            <v>2.0020410407538263</v>
-          </cell>
           <cell r="B104">
             <v>102</v>
           </cell>
         </row>
         <row r="105">
-          <cell r="A105">
-            <v>2.0020610612643361</v>
-          </cell>
           <cell r="B105">
             <v>103</v>
           </cell>
         </row>
         <row r="106">
-          <cell r="A106">
-            <v>2.0020810819750521</v>
-          </cell>
           <cell r="B106">
             <v>104</v>
           </cell>
         </row>
         <row r="107">
-          <cell r="A107">
-            <v>2.0021011028859763</v>
-          </cell>
           <cell r="B107">
             <v>105</v>
           </cell>
         </row>
         <row r="108">
-          <cell r="A108">
-            <v>2.0021211239971106</v>
-          </cell>
           <cell r="B108">
             <v>106</v>
           </cell>
         </row>
         <row r="109">
-          <cell r="A109">
-            <v>2.0021411453084568</v>
-          </cell>
           <cell r="B109">
             <v>107</v>
           </cell>
         </row>
         <row r="110">
-          <cell r="A110">
-            <v>2.0021611668200174</v>
-          </cell>
           <cell r="B110">
             <v>108</v>
           </cell>
         </row>
         <row r="111">
-          <cell r="A111">
-            <v>2.0021811885317939</v>
-          </cell>
           <cell r="B111">
             <v>109</v>
           </cell>
         </row>
         <row r="112">
-          <cell r="A112">
-            <v>2.0022012104437885</v>
-          </cell>
           <cell r="B112">
             <v>110</v>
           </cell>
         </row>
         <row r="113">
-          <cell r="A113">
-            <v>2.0022212325560034</v>
-          </cell>
           <cell r="B113">
             <v>111</v>
           </cell>
         </row>
         <row r="114">
-          <cell r="A114">
-            <v>2.0022412548684403</v>
-          </cell>
           <cell r="B114">
             <v>112</v>
           </cell>
         </row>
         <row r="115">
-          <cell r="A115">
-            <v>2.0022612773811015</v>
-          </cell>
           <cell r="B115">
             <v>113</v>
           </cell>
         </row>
         <row r="116">
-          <cell r="A116">
-            <v>2.0022813000939887</v>
-          </cell>
           <cell r="B116">
             <v>114</v>
           </cell>
         </row>
         <row r="117">
-          <cell r="A117">
-            <v>2.0023013230071043</v>
-          </cell>
           <cell r="B117">
             <v>115</v>
           </cell>
         </row>
         <row r="118">
-          <cell r="A118">
-            <v>2.0023213461204494</v>
-          </cell>
           <cell r="B118">
             <v>116</v>
           </cell>
         </row>
         <row r="119">
-          <cell r="A119">
-            <v>2.0023413694340273</v>
-          </cell>
           <cell r="B119">
             <v>117</v>
           </cell>
         </row>
         <row r="120">
-          <cell r="A120">
-            <v>2.0023613929478388</v>
-          </cell>
           <cell r="B120">
             <v>118</v>
           </cell>
         </row>
         <row r="121">
-          <cell r="A121">
-            <v>2.002381416661887</v>
-          </cell>
           <cell r="B121">
             <v>119</v>
           </cell>
         </row>
         <row r="122">
-          <cell r="A122">
-            <v>2.0024014405761728</v>
-          </cell>
           <cell r="B122">
             <v>120</v>
           </cell>
         </row>
         <row r="123">
-          <cell r="A123">
-            <v>2.0024214646906988</v>
-          </cell>
           <cell r="B123">
             <v>121</v>
           </cell>
         </row>
         <row r="124">
-          <cell r="A124">
-            <v>2.0024414890054674</v>
-          </cell>
           <cell r="B124">
             <v>122</v>
           </cell>
         </row>
         <row r="125">
-          <cell r="A125">
-            <v>2.0024615135204797</v>
-          </cell>
           <cell r="B125">
             <v>123</v>
           </cell>
         </row>
         <row r="126">
-          <cell r="A126">
-            <v>2.0024815382357386</v>
-          </cell>
           <cell r="B126">
             <v>124</v>
           </cell>
         </row>
         <row r="127">
-          <cell r="A127">
-            <v>2.0025015631512453</v>
-          </cell>
           <cell r="B127">
             <v>125</v>
           </cell>
         </row>
         <row r="128">
-          <cell r="A128">
-            <v>2.002521588267002</v>
-          </cell>
           <cell r="B128">
             <v>126</v>
           </cell>
         </row>
         <row r="129">
-          <cell r="A129">
-            <v>2.002541613583011</v>
-          </cell>
           <cell r="B129">
             <v>127</v>
           </cell>
         </row>
         <row r="130">
-          <cell r="A130">
-            <v>2.0025616390992744</v>
-          </cell>
           <cell r="B130">
             <v>128</v>
           </cell>
         </row>
         <row r="131">
-          <cell r="A131">
-            <v>2.0025816648157937</v>
-          </cell>
           <cell r="B131">
             <v>129</v>
           </cell>
         </row>
         <row r="132">
-          <cell r="A132">
-            <v>2.0026016907325714</v>
-          </cell>
           <cell r="B132">
             <v>130</v>
           </cell>
         </row>
         <row r="133">
-          <cell r="A133">
-            <v>2.002621716849609</v>
-          </cell>
           <cell r="B133">
             <v>131</v>
           </cell>
         </row>
         <row r="134">
-          <cell r="A134">
-            <v>2.002641743166909</v>
-          </cell>
           <cell r="B134">
             <v>132</v>
           </cell>
         </row>
         <row r="135">
-          <cell r="A135">
-            <v>2.0026617696844733</v>
-          </cell>
           <cell r="B135">
             <v>133</v>
           </cell>
         </row>
         <row r="136">
-          <cell r="A136">
-            <v>2.0026817964023036</v>
-          </cell>
           <cell r="B136">
             <v>134</v>
           </cell>
         </row>
         <row r="137">
-          <cell r="A137">
-            <v>2.0027018233204017</v>
-          </cell>
           <cell r="B137">
             <v>135</v>
           </cell>
         </row>
         <row r="138">
-          <cell r="A138">
-            <v>2.0027218504387707</v>
-          </cell>
           <cell r="B138">
             <v>136</v>
           </cell>
         </row>
         <row r="139">
-          <cell r="A139">
-            <v>2.0027418777574115</v>
-          </cell>
           <cell r="B139">
             <v>137</v>
           </cell>
         </row>
         <row r="140">
-          <cell r="A140">
-            <v>2.0027619052763264</v>
-          </cell>
           <cell r="B140">
             <v>138</v>
           </cell>
         </row>
         <row r="141">
-          <cell r="A141">
-            <v>2.0027819329955174</v>
-          </cell>
           <cell r="B141">
             <v>139</v>
           </cell>
         </row>
         <row r="142">
-          <cell r="A142">
-            <v>2.002801960914987</v>
-          </cell>
           <cell r="B142">
             <v>140</v>
           </cell>
         </row>
         <row r="143">
-          <cell r="A143">
-            <v>2.0028219890347363</v>
-          </cell>
           <cell r="B143">
             <v>141</v>
           </cell>
         </row>
         <row r="144">
-          <cell r="A144">
-            <v>2.0028420173547681</v>
-          </cell>
           <cell r="B144">
             <v>142</v>
           </cell>
         </row>
         <row r="145">
-          <cell r="A145">
-            <v>2.0028620458750841</v>
-          </cell>
           <cell r="B145">
             <v>143</v>
           </cell>
         </row>
         <row r="146">
-          <cell r="A146">
-            <v>2.0028820745956866</v>
-          </cell>
           <cell r="B146">
             <v>144</v>
           </cell>
         </row>
         <row r="147">
-          <cell r="A147">
-            <v>2.0029021035165768</v>
-          </cell>
           <cell r="B147">
             <v>145</v>
           </cell>
         </row>
         <row r="148">
-          <cell r="A148">
-            <v>2.0029221326377575</v>
-          </cell>
           <cell r="B148">
             <v>146</v>
           </cell>
         </row>
         <row r="149">
-          <cell r="A149">
-            <v>2.00294216195923</v>
-          </cell>
           <cell r="B149">
             <v>147</v>
           </cell>
         </row>
         <row r="150">
-          <cell r="A150">
-            <v>2.0029621914809974</v>
-          </cell>
           <cell r="B150">
             <v>148</v>
           </cell>
         </row>
         <row r="151">
-          <cell r="A151">
-            <v>2.0029822212030606</v>
-          </cell>
           <cell r="B151">
             <v>149</v>
           </cell>
         </row>
         <row r="152">
-          <cell r="A152">
-            <v>2.0030022511254222</v>
-          </cell>
           <cell r="B152">
             <v>150</v>
           </cell>
         </row>
         <row r="153">
-          <cell r="A153">
-            <v>2.0030222812480836</v>
-          </cell>
           <cell r="B153">
             <v>151</v>
           </cell>
         </row>
         <row r="154">
-          <cell r="A154">
-            <v>2.0030423115710478</v>
-          </cell>
           <cell r="B154">
             <v>152</v>
           </cell>
         </row>
         <row r="155">
-          <cell r="A155">
-            <v>2.0030623420943159</v>
-          </cell>
           <cell r="B155">
             <v>153</v>
           </cell>
         </row>
         <row r="156">
-          <cell r="A156">
-            <v>2.0030823728178904</v>
-          </cell>
           <cell r="B156">
             <v>154</v>
           </cell>
         </row>
         <row r="157">
-          <cell r="A157">
-            <v>2.0031024037417726</v>
-          </cell>
           <cell r="B157">
             <v>155</v>
           </cell>
         </row>
         <row r="158">
-          <cell r="A158">
-            <v>2.0031224348659658</v>
-          </cell>
           <cell r="B158">
             <v>156</v>
           </cell>
         </row>
         <row r="159">
-          <cell r="A159">
-            <v>2.0031424661904706</v>
-          </cell>
           <cell r="B159">
             <v>157</v>
           </cell>
         </row>
         <row r="160">
-          <cell r="A160">
-            <v>2.00316249771529</v>
-          </cell>
           <cell r="B160">
             <v>158</v>
           </cell>
         </row>
         <row r="161">
-          <cell r="A161">
-            <v>2.003182529440426</v>
-          </cell>
           <cell r="B161">
             <v>159</v>
           </cell>
         </row>
         <row r="162">
-          <cell r="A162">
-            <v>2.0032025613658795</v>
-          </cell>
           <cell r="B162">
             <v>160</v>
           </cell>
         </row>
         <row r="163">
-          <cell r="A163">
-            <v>2.0032225934916537</v>
-          </cell>
           <cell r="B163">
             <v>161</v>
           </cell>
         </row>
         <row r="164">
-          <cell r="A164">
-            <v>2.0032426258177503</v>
-          </cell>
           <cell r="B164">
             <v>162</v>
           </cell>
         </row>
         <row r="165">
-          <cell r="A165">
-            <v>2.0032626583441706</v>
-          </cell>
           <cell r="B165">
             <v>163</v>
           </cell>
         </row>
         <row r="166">
-          <cell r="A166">
-            <v>2.0032826910709178</v>
-          </cell>
           <cell r="B166">
             <v>164</v>
           </cell>
         </row>
         <row r="167">
-          <cell r="A167">
-            <v>2.0033027239979928</v>
-          </cell>
           <cell r="B167">
             <v>165</v>
           </cell>
         </row>
         <row r="168">
-          <cell r="A168">
-            <v>2.0033227571253982</v>
-          </cell>
           <cell r="B168">
             <v>166</v>
           </cell>
         </row>
         <row r="169">
-          <cell r="A169">
-            <v>2.0033427904531362</v>
-          </cell>
           <cell r="B169">
             <v>167</v>
           </cell>
         </row>
         <row r="170">
-          <cell r="A170">
-            <v>2.0033628239812082</v>
-          </cell>
           <cell r="B170">
             <v>168</v>
           </cell>
         </row>
         <row r="171">
-          <cell r="A171">
-            <v>2.0033828577096164</v>
-          </cell>
           <cell r="B171">
             <v>169</v>
           </cell>
         </row>
         <row r="172">
-          <cell r="A172">
-            <v>2.003402891638363</v>
-          </cell>
           <cell r="B172">
             <v>170</v>
           </cell>
         </row>
         <row r="173">
-          <cell r="A173">
-            <v>2.0034229257674498</v>
-          </cell>
           <cell r="B173">
             <v>171</v>
           </cell>
         </row>
         <row r="174">
-          <cell r="A174">
-            <v>2.0034429600968791</v>
-          </cell>
           <cell r="B174">
             <v>172</v>
           </cell>
         </row>
         <row r="175">
-          <cell r="A175">
-            <v>2.0034629946266524</v>
-          </cell>
           <cell r="B175">
             <v>173</v>
           </cell>
         </row>
         <row r="176">
-          <cell r="A176">
-            <v>2.0034830293567722</v>
-          </cell>
           <cell r="B176">
             <v>174</v>
           </cell>
         </row>
         <row r="177">
-          <cell r="A177">
-            <v>2.0035030642872402</v>
-          </cell>
           <cell r="B177">
             <v>175</v>
           </cell>
         </row>
         <row r="178">
-          <cell r="A178">
-            <v>2.0035230994180586</v>
-          </cell>
           <cell r="B178">
             <v>176</v>
           </cell>
         </row>
         <row r="179">
-          <cell r="A179">
-            <v>2.0035431347492292</v>
-          </cell>
           <cell r="B179">
             <v>177</v>
           </cell>
         </row>
         <row r="180">
-          <cell r="A180">
-            <v>2.0035631702807541</v>
-          </cell>
           <cell r="B180">
             <v>178</v>
           </cell>
         </row>
         <row r="181">
-          <cell r="A181">
-            <v>2.0035832060126353</v>
-          </cell>
           <cell r="B181">
             <v>179</v>
           </cell>
         </row>
         <row r="182">
-          <cell r="A182">
-            <v>2.0036032419448753</v>
-          </cell>
           <cell r="B182">
             <v>180</v>
           </cell>
         </row>
         <row r="183">
-          <cell r="A183">
-            <v>2.003623278077475</v>
-          </cell>
           <cell r="B183">
             <v>181</v>
           </cell>
         </row>
         <row r="184">
-          <cell r="A184">
-            <v>2.0036433144104375</v>
-          </cell>
           <cell r="B184">
             <v>182</v>
           </cell>
         </row>
         <row r="185">
-          <cell r="A185">
-            <v>2.0036633509437638</v>
-          </cell>
           <cell r="B185">
             <v>183</v>
           </cell>
         </row>
         <row r="186">
-          <cell r="A186">
-            <v>2.0036833876774569</v>
-          </cell>
           <cell r="B186">
             <v>184</v>
           </cell>
         </row>
         <row r="187">
-          <cell r="A187">
-            <v>2.0037034246115182</v>
-          </cell>
           <cell r="B187">
             <v>185</v>
           </cell>
         </row>
         <row r="188">
-          <cell r="A188">
-            <v>2.0037234617459498</v>
-          </cell>
           <cell r="B188">
             <v>186</v>
           </cell>
         </row>
         <row r="189">
-          <cell r="A189">
-            <v>2.0037434990807537</v>
-          </cell>
           <cell r="B189">
             <v>187</v>
           </cell>
         </row>
         <row r="190">
-          <cell r="A190">
-            <v>2.0037635366159319</v>
-          </cell>
           <cell r="B190">
             <v>188</v>
           </cell>
         </row>
         <row r="191">
-          <cell r="A191">
-            <v>2.0037835743514867</v>
-          </cell>
           <cell r="B191">
             <v>189</v>
           </cell>
         </row>
         <row r="192">
-          <cell r="A192">
-            <v>2.0038036122874199</v>
-          </cell>
           <cell r="B192">
             <v>190</v>
           </cell>
         </row>
         <row r="193">
-          <cell r="A193">
-            <v>2.0038236504237332</v>
-          </cell>
           <cell r="B193">
             <v>191</v>
           </cell>
         </row>
         <row r="194">
-          <cell r="A194">
-            <v>2.003843688760429</v>
-          </cell>
           <cell r="B194">
             <v>192</v>
           </cell>
         </row>
         <row r="195">
-          <cell r="A195">
-            <v>2.0038637272975088</v>
-          </cell>
           <cell r="B195">
             <v>193</v>
           </cell>
         </row>
         <row r="196">
-          <cell r="A196">
-            <v>2.0038837660349755</v>
-          </cell>
           <cell r="B196">
             <v>194</v>
           </cell>
         </row>
         <row r="197">
-          <cell r="A197">
-            <v>2.0039038049728304</v>
-          </cell>
           <cell r="B197">
             <v>195</v>
           </cell>
         </row>
         <row r="198">
-          <cell r="A198">
-            <v>2.0039238441110756</v>
-          </cell>
           <cell r="B198">
             <v>196</v>
           </cell>
         </row>
         <row r="199">
-          <cell r="A199">
-            <v>2.0039438834497134</v>
-          </cell>
           <cell r="B199">
             <v>197</v>
           </cell>
         </row>
         <row r="200">
-          <cell r="A200">
-            <v>2.0039639229887451</v>
-          </cell>
           <cell r="B200">
             <v>198</v>
           </cell>
         </row>
         <row r="201">
-          <cell r="A201">
-            <v>2.0039839627281739</v>
-          </cell>
           <cell r="B201">
             <v>199</v>
           </cell>
         </row>
         <row r="202">
-          <cell r="A202">
-            <v>2.0040040026680006</v>
-          </cell>
           <cell r="B202">
             <v>200</v>
           </cell>
@@ -6178,13 +5578,13 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>